<commit_message>
Completed analysis, need to draft up commentary.
</commit_message>
<xml_diff>
--- a/ECOM90024 - FEB/Assignment 1/applerev.xlsx
+++ b/ECOM90024 - FEB/Assignment 1/applerev.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10312"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27328"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://unimelbcloud-my.sharepoint.com/personal/jonathan_thong_unimelb_edu_au/Documents/Forecasting in Economics and Business - S12023/Assignment 1/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/16fd880609b67c05/Desktop/git/mae_unimelb/ECOM90024 - FEB/Assignment 1/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="2" documentId="8_{85DFD23D-F353-064E-965C-0A30ABDD86CE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{53EF5BE2-C35F-3F4D-B064-7EA4BFA06A9F}"/>
+  <xr:revisionPtr revIDLastSave="4" documentId="8_{85DFD23D-F353-064E-965C-0A30ABDD86CE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F731F1E6-F596-44C5-9AA2-FF49B39275CE}"/>
   <bookViews>
-    <workbookView xWindow="11980" yWindow="5900" windowWidth="27640" windowHeight="16940" xr2:uid="{9E190F83-D5EE-B642-9108-D9C644A04DAA}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{9E190F83-D5EE-B642-9108-D9C644A04DAA}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -247,9 +247,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -287,7 +287,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -393,7 +393,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -535,7 +535,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -544,12 +544,12 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1700E75A-170C-8742-A1C6-5C58132049C3}">
   <dimension ref="A1:B51"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="11.19921875" defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="16.33203125" customWidth="1"/>
+    <col min="1" max="1" width="22.5" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -557,7 +557,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>2</v>
       </c>
@@ -565,7 +565,7 @@
         <v>20.34</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>3</v>
       </c>
@@ -573,7 +573,7 @@
         <v>26.74</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>4</v>
       </c>
@@ -581,7 +581,7 @@
         <v>24.67</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>5</v>
       </c>
@@ -589,7 +589,7 @@
         <v>28.57</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>6</v>
       </c>
@@ -597,7 +597,7 @@
         <v>28.27</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>7</v>
       </c>
@@ -605,7 +605,7 @@
         <v>46.33</v>
       </c>
     </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>8</v>
       </c>
@@ -613,7 +613,7 @@
         <v>39.19</v>
       </c>
     </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>9</v>
       </c>
@@ -621,7 +621,7 @@
         <v>35.020000000000003</v>
       </c>
     </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>10</v>
       </c>
@@ -629,7 +629,7 @@
         <v>35.97</v>
       </c>
     </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>11</v>
       </c>
@@ -637,7 +637,7 @@
         <v>54.51</v>
       </c>
     </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>12</v>
       </c>
@@ -645,7 +645,7 @@
         <v>43.6</v>
       </c>
     </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>13</v>
       </c>
@@ -653,7 +653,7 @@
         <v>35.32</v>
       </c>
     </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
         <v>14</v>
       </c>
@@ -661,7 +661,7 @@
         <v>37.47</v>
       </c>
     </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
         <v>15</v>
       </c>
@@ -669,7 +669,7 @@
         <v>57.59</v>
       </c>
     </row>
-    <row r="16" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
         <v>16</v>
       </c>
@@ -677,7 +677,7 @@
         <v>45.65</v>
       </c>
     </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
         <v>17</v>
       </c>
@@ -685,7 +685,7 @@
         <v>37.43</v>
       </c>
     </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
         <v>18</v>
       </c>
@@ -693,7 +693,7 @@
         <v>42.12</v>
       </c>
     </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
         <v>19</v>
       </c>
@@ -701,7 +701,7 @@
         <v>74.599999999999994</v>
       </c>
     </row>
-    <row r="20" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
         <v>20</v>
       </c>
@@ -709,7 +709,7 @@
         <v>58.01</v>
       </c>
     </row>
-    <row r="21" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
         <v>21</v>
       </c>
@@ -717,7 +717,7 @@
         <v>49.6</v>
       </c>
     </row>
-    <row r="22" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
         <v>22</v>
       </c>
@@ -725,7 +725,7 @@
         <v>51.5</v>
       </c>
     </row>
-    <row r="23" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
         <v>23</v>
       </c>
@@ -733,7 +733,7 @@
         <v>75.87</v>
       </c>
     </row>
-    <row r="24" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
         <v>24</v>
       </c>
@@ -741,7 +741,7 @@
         <v>50.56</v>
       </c>
     </row>
-    <row r="25" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
         <v>25</v>
       </c>
@@ -749,7 +749,7 @@
         <v>42.36</v>
       </c>
     </row>
-    <row r="26" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
         <v>26</v>
       </c>
@@ -757,7 +757,7 @@
         <v>46.85</v>
       </c>
     </row>
-    <row r="27" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
         <v>27</v>
       </c>
@@ -765,7 +765,7 @@
         <v>78.349999999999994</v>
       </c>
     </row>
-    <row r="28" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
         <v>28</v>
       </c>
@@ -773,7 +773,7 @@
         <v>52.9</v>
       </c>
     </row>
-    <row r="29" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
         <v>29</v>
       </c>
@@ -781,7 +781,7 @@
         <v>45.41</v>
       </c>
     </row>
-    <row r="30" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A30" t="s">
         <v>30</v>
       </c>
@@ -789,7 +789,7 @@
         <v>52.58</v>
       </c>
     </row>
-    <row r="31" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A31" t="s">
         <v>31</v>
       </c>
@@ -797,7 +797,7 @@
         <v>88.29</v>
       </c>
     </row>
-    <row r="32" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="32" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A32" t="s">
         <v>32</v>
       </c>
@@ -805,7 +805,7 @@
         <v>61.14</v>
       </c>
     </row>
-    <row r="33" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="33" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A33" t="s">
         <v>33</v>
       </c>
@@ -813,7 +813,7 @@
         <v>53.26</v>
       </c>
     </row>
-    <row r="34" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="34" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A34" t="s">
         <v>34</v>
       </c>
@@ -821,7 +821,7 @@
         <v>62.9</v>
       </c>
     </row>
-    <row r="35" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="35" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A35" t="s">
         <v>35</v>
       </c>
@@ -829,7 +829,7 @@
         <v>84.31</v>
       </c>
     </row>
-    <row r="36" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="36" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A36" t="s">
         <v>36</v>
       </c>
@@ -837,7 +837,7 @@
         <v>58.02</v>
       </c>
     </row>
-    <row r="37" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="37" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A37" t="s">
         <v>37</v>
       </c>
@@ -845,7 +845,7 @@
         <v>53.81</v>
       </c>
     </row>
-    <row r="38" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="38" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A38" t="s">
         <v>38</v>
       </c>
@@ -853,7 +853,7 @@
         <v>64.040000000000006</v>
       </c>
     </row>
-    <row r="39" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="39" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A39" t="s">
         <v>39</v>
       </c>
@@ -861,7 +861,7 @@
         <v>91.82</v>
       </c>
     </row>
-    <row r="40" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="40" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A40" t="s">
         <v>40</v>
       </c>
@@ -869,7 +869,7 @@
         <v>58.31</v>
       </c>
     </row>
-    <row r="41" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="41" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A41" t="s">
         <v>41</v>
       </c>
@@ -877,7 +877,7 @@
         <v>59.68</v>
       </c>
     </row>
-    <row r="42" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="42" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A42" t="s">
         <v>42</v>
       </c>
@@ -885,7 +885,7 @@
         <v>64.7</v>
       </c>
     </row>
-    <row r="43" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="43" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A43" t="s">
         <v>43</v>
       </c>
@@ -893,7 +893,7 @@
         <v>111.44</v>
       </c>
     </row>
-    <row r="44" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="44" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A44" t="s">
         <v>44</v>
       </c>
@@ -901,7 +901,7 @@
         <v>89.58</v>
       </c>
     </row>
-    <row r="45" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="45" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A45" t="s">
         <v>45</v>
       </c>
@@ -909,7 +909,7 @@
         <v>81.430000000000007</v>
       </c>
     </row>
-    <row r="46" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="46" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A46" t="s">
         <v>46</v>
       </c>
@@ -917,7 +917,7 @@
         <v>83.36</v>
       </c>
     </row>
-    <row r="47" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="47" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A47" t="s">
         <v>47</v>
       </c>
@@ -925,7 +925,7 @@
         <v>123.94</v>
       </c>
     </row>
-    <row r="48" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="48" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A48" t="s">
         <v>48</v>
       </c>
@@ -933,7 +933,7 @@
         <v>97.28</v>
       </c>
     </row>
-    <row r="49" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="49" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A49" t="s">
         <v>49</v>
       </c>
@@ -941,7 +941,7 @@
         <v>82.96</v>
       </c>
     </row>
-    <row r="50" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="50" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A50" t="s">
         <v>50</v>
       </c>
@@ -949,7 +949,7 @@
         <v>90.15</v>
       </c>
     </row>
-    <row r="51" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="51" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A51" t="s">
         <v>51</v>
       </c>

</xml_diff>